<commit_message>
Created PdfService class for reading PDF files and extracting data from it.
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -36,26 +36,8 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
-Canadian-United States-Mexico Agreement (CUSMA)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="18"/>
-        <color rgb="FF076DD3"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Trada Mexico Estados Unido Canada (T-MEC)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="18"/>
-        <color rgb="FF076DD3"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
+Canadian-United States-Mexico Agreement (CUSMA)
+Trada Mexico Estados Unido Canada (T-MEC)
 Unites States-Mexico-Canada Agreement (USMCA)</t>
     </r>
   </si>

</xml_diff>